<commit_message>
docs: update voice command protocol table
</commit_message>
<xml_diff>
--- a/docs/语音交互模块/2.2 命令词播报词协议列表.xlsx
+++ b/docs/语音交互模块/2.2 命令词播报词协议列表.xlsx
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="370">
   <si>
     <t>语义标签</t>
   </si>
@@ -1224,6 +1224,30 @@
   </si>
   <si>
     <t>2、如果某个命令词的识别不够灵敏，可在页面上更改该命令词的置信度阈值提高其识别灵敏度（非自动优化模式）；也可以增加同一语义的命令词以提高其识别泛化性</t>
+  </si>
+  <si>
+    <t>你好，有什么可以帮您</t>
+  </si>
+  <si>
+    <t>我是一朵会追光的闲聊花，可以陪你说说话</t>
+  </si>
+  <si>
+    <t>我有点累</t>
+  </si>
+  <si>
+    <t>那就休息一下吧，喝口水，看看远处</t>
+  </si>
+  <si>
+    <t>今天开心</t>
+  </si>
+  <si>
+    <t>太好啦，希望这份开心一直陪着你</t>
+  </si>
+  <si>
+    <t>我要走了</t>
+  </si>
+  <si>
+    <t>好的，待会儿见，我会继续面朝阳光</t>
   </si>
 </sst>
 </file>
@@ -2326,7 +2350,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr/>
   <dimension ref="A1:J152"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
@@ -3234,7 +3258,7 @@
         <v>1</v>
       </c>
       <c r="D40" t="s">
-        <v>107</v>
+        <v>362</v>
       </c>
       <c r="E40" t="s">
         <v>19</v>
@@ -3259,7 +3283,7 @@
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="E41" t="s">
         <v>19</v>
@@ -3278,13 +3302,13 @@
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>112</v>
+        <v>364</v>
       </c>
       <c r="C42" t="s">
         <v>1</v>
       </c>
       <c r="D42" t="s">
-        <v>113</v>
+        <v>365</v>
       </c>
       <c r="E42" t="s">
         <v>19</v>
@@ -3303,13 +3327,13 @@
         <v>39</v>
       </c>
       <c r="B43" t="s">
-        <v>115</v>
+        <v>366</v>
       </c>
       <c r="C43" t="s">
         <v>1</v>
       </c>
       <c r="D43" t="s">
-        <v>60</v>
+        <v>367</v>
       </c>
       <c r="E43" t="s">
         <v>19</v>
@@ -3328,13 +3352,13 @@
         <v>40</v>
       </c>
       <c r="B44" t="s">
-        <v>117</v>
+        <v>368</v>
       </c>
       <c r="C44" t="s">
         <v>1</v>
       </c>
       <c r="D44" t="s">
-        <v>65</v>
+        <v>369</v>
       </c>
       <c r="E44" t="s">
         <v>19</v>
@@ -5810,7 +5834,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
-  <legacyDrawing r:id="rId2"/>
+  <legacyDrawing ns1:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>